<commit_message>
NewHire Ireland Testcase 10%
</commit_message>
<xml_diff>
--- a/Data/Hires/TestDataSloveniaMKv1.xlsx
+++ b/Data/Hires/TestDataSloveniaMKv1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{3BDC4FFC-8847-4F75-A8A0-26E78603E1E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{010A94B2-E573-40BF-B6FF-36154ED89136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="912" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="191">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -244,190 +244,190 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10698062</t>
+    <t>Test failed for 'Eden Rogahn' Employee: Errors and AlertsErrorsPage ErrorSorry, the data you requested could not be found. Please refresh your page.ErrorAllowance Amount is required.ErrorAllowance Amount is required.Alerts &amp; find failed Screenshot Path:-&gt;H:\WorkdaySuite_Playwright_MK/WorkdayFailedScreenshot/2025-03-25T10-19-24-088Z.png</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>795 Store Management (Zogop Dogegy (On Leave) (10185858))</t>
+  </si>
+  <si>
+    <t>Slovenia</t>
+  </si>
+  <si>
+    <t>Eden</t>
+  </si>
+  <si>
+    <t>Rogahn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">070-417-626 </t>
+  </si>
+  <si>
+    <t>Landline</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>Automation Street Name</t>
+  </si>
+  <si>
+    <t>Ljubljana</t>
+  </si>
+  <si>
+    <t>Street Address</t>
+  </si>
+  <si>
+    <t>Test@email.com</t>
+  </si>
+  <si>
+    <t>New Hire</t>
+  </si>
+  <si>
+    <t>Auto 9148281</t>
+  </si>
+  <si>
+    <t>Permanent</t>
+  </si>
+  <si>
+    <t>Store Manager_NEW</t>
+  </si>
+  <si>
+    <t>Full time</t>
+  </si>
+  <si>
+    <t>Salary</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>5 Days (Slovenia)</t>
+  </si>
+  <si>
+    <t>0- Ne gre za zaposlitev po ZUTD-A ali ZIUPTDSV</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Collective Agreement - Slovenia (01/01/1900 - )</t>
+  </si>
+  <si>
+    <t>Asistent v prodaji</t>
+  </si>
+  <si>
+    <t>IV.</t>
+  </si>
+  <si>
+    <t>Unique Master Citizen Number</t>
+  </si>
+  <si>
+    <t>01/01/1999</t>
+  </si>
+  <si>
+    <t>01/01/2045</t>
+  </si>
+  <si>
+    <t>Slovenia Tax Number</t>
+  </si>
+  <si>
+    <t>01/01/2041</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Citizen (Slovenia)</t>
+  </si>
+  <si>
+    <t>TestBankOFSlovenia</t>
+  </si>
+  <si>
+    <t>Checking</t>
+  </si>
+  <si>
+    <t>SI56 2633 0001 2039 086</t>
+  </si>
+  <si>
+    <t>Grun Frun</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>SVN Monthly</t>
+  </si>
+  <si>
+    <t>Test2</t>
+  </si>
+  <si>
+    <t>10698135</t>
   </si>
   <si>
     <t>Passed</t>
   </si>
   <si>
+    <t>795 Recruitment (Zosig Depazi (10280602))</t>
+  </si>
+  <si>
+    <t>Carmel</t>
+  </si>
+  <si>
+    <t>Hane</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Retail Assistant_NEW</t>
+  </si>
+  <si>
+    <t>94 Retail Operatives</t>
+  </si>
+  <si>
+    <t>01 Accessories</t>
+  </si>
+  <si>
+    <t>Test3</t>
+  </si>
+  <si>
+    <t>795 Retail Team 1 (Zogop Dogegy (10185858) (Inherited))</t>
+  </si>
+  <si>
+    <t>Jensen</t>
+  </si>
+  <si>
+    <t>O'Connell</t>
+  </si>
+  <si>
+    <t>Fixed Term (Fixed Term)</t>
+  </si>
+  <si>
+    <t>Part time</t>
+  </si>
+  <si>
+    <t>3 Days (Slovenia)</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Test4</t>
+  </si>
+  <si>
     <t>795 Store Management (Zogop Dogegy (10185858))</t>
   </si>
   <si>
-    <t>Slovenia</t>
-  </si>
-  <si>
-    <t>Parker</t>
-  </si>
-  <si>
-    <t>Halvorson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">070-417-626 </t>
-  </si>
-  <si>
-    <t>Landline</t>
-  </si>
-  <si>
-    <t>Home</t>
-  </si>
-  <si>
-    <t>Automation Street Name</t>
-  </si>
-  <si>
-    <t>Ljubljana</t>
-  </si>
-  <si>
-    <t>Street Address</t>
-  </si>
-  <si>
-    <t>Test@email.com</t>
-  </si>
-  <si>
-    <t>New Hire</t>
-  </si>
-  <si>
-    <t>Auto 95021107</t>
-  </si>
-  <si>
-    <t>Permanent</t>
-  </si>
-  <si>
-    <t>Store Manager_NEW</t>
-  </si>
-  <si>
-    <t>Full time</t>
-  </si>
-  <si>
-    <t>Salary</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>5 Days (Slovenia)</t>
-  </si>
-  <si>
-    <t>0- Ne gre za zaposlitev po ZUTD-A ali ZIUPTDSV</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Collective Agreement - Slovenia (01/01/1900 - )</t>
-  </si>
-  <si>
-    <t>Asistent v prodaji</t>
-  </si>
-  <si>
-    <t>IV.</t>
-  </si>
-  <si>
-    <t>Unique Master Citizen Number</t>
-  </si>
-  <si>
-    <t>01/01/1999</t>
-  </si>
-  <si>
-    <t>01/01/2045</t>
-  </si>
-  <si>
-    <t>Slovenia Tax Number</t>
-  </si>
-  <si>
-    <t>01/01/2041</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>Citizen (Slovenia)</t>
-  </si>
-  <si>
-    <t>TestBankOFSlovenia</t>
-  </si>
-  <si>
-    <t>Checking</t>
-  </si>
-  <si>
-    <t>SI56 2633 0001 2039 086</t>
-  </si>
-  <si>
-    <t>Grun Frun</t>
-  </si>
-  <si>
-    <t>Standard</t>
-  </si>
-  <si>
-    <t>SVN Monthly</t>
-  </si>
-  <si>
-    <t>Test2</t>
-  </si>
-  <si>
-    <t>10698063</t>
-  </si>
-  <si>
-    <t>795 Recruitment (Zosig Depazi (10280602))</t>
-  </si>
-  <si>
-    <t>Mittie</t>
-  </si>
-  <si>
-    <t>Tillman</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Retail Assistant_NEW</t>
-  </si>
-  <si>
-    <t>94 Retail Operatives</t>
-  </si>
-  <si>
-    <t>01 Accessories</t>
-  </si>
-  <si>
-    <t>Test3</t>
-  </si>
-  <si>
-    <t>10698065</t>
-  </si>
-  <si>
-    <t>795 Retail Team 1 (Zogop Dogegy (10185858) (Inherited))</t>
-  </si>
-  <si>
-    <t>Aurore</t>
-  </si>
-  <si>
-    <t>Kreiger</t>
-  </si>
-  <si>
-    <t>Fixed Term (Fixed Term)</t>
-  </si>
-  <si>
-    <t>Part time</t>
-  </si>
-  <si>
-    <t>3 Days (Slovenia)</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>Test4</t>
-  </si>
-  <si>
-    <t>10698066</t>
-  </si>
-  <si>
-    <t>Antwon</t>
-  </si>
-  <si>
-    <t>Johns</t>
-  </si>
-  <si>
-    <t>Auto 5780199</t>
+    <t>Jairo</t>
+  </si>
+  <si>
+    <t>Gerhold</t>
+  </si>
+  <si>
+    <t>Auto 13582723</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -439,13 +439,10 @@
     <t>Test5</t>
   </si>
   <si>
-    <t>10698068</t>
-  </si>
-  <si>
-    <t>Rebeka</t>
-  </si>
-  <si>
-    <t>Watsica</t>
+    <t>Fritz</t>
+  </si>
+  <si>
+    <t>Bayer</t>
   </si>
   <si>
     <t>In-Store Visual Merchandising Assistant_NEW</t>
@@ -457,16 +454,13 @@
     <t>Test6</t>
   </si>
   <si>
-    <t>10698070</t>
-  </si>
-  <si>
-    <t>Aron</t>
-  </si>
-  <si>
-    <t>Armstrong-McKenzie</t>
-  </si>
-  <si>
-    <t>Auto 7225502</t>
+    <t>Christopher</t>
+  </si>
+  <si>
+    <t>Schuppe</t>
+  </si>
+  <si>
+    <t>Auto 56790541</t>
   </si>
   <si>
     <t>Strokovni sodelavec v kadrovski službi</t>
@@ -478,16 +472,13 @@
     <t>Test7</t>
   </si>
   <si>
-    <t>10698072</t>
-  </si>
-  <si>
-    <t>Uriah</t>
-  </si>
-  <si>
-    <t>Medhurst</t>
-  </si>
-  <si>
-    <t>Auto 66154525</t>
+    <t>Bridget</t>
+  </si>
+  <si>
+    <t>Moen</t>
+  </si>
+  <si>
+    <t>Auto 67393007</t>
   </si>
   <si>
     <t>Assistant Store Manager_NEW</t>
@@ -496,16 +487,13 @@
     <t>Test8</t>
   </si>
   <si>
-    <t>10698073</t>
-  </si>
-  <si>
-    <t>Abby</t>
-  </si>
-  <si>
-    <t>Becker</t>
-  </si>
-  <si>
-    <t>Auto 6021389</t>
+    <t>Abdullah</t>
+  </si>
+  <si>
+    <t>Dickinson</t>
+  </si>
+  <si>
+    <t>Auto 39443903</t>
   </si>
   <si>
     <t>Department Manager_NEW</t>
@@ -514,16 +502,13 @@
     <t>Test9</t>
   </si>
   <si>
-    <t>10698074</t>
-  </si>
-  <si>
-    <t>Lindsey</t>
-  </si>
-  <si>
-    <t>Hagenes</t>
-  </si>
-  <si>
-    <t>Auto 51830818</t>
+    <t>Christa</t>
+  </si>
+  <si>
+    <t>Balistreri</t>
+  </si>
+  <si>
+    <t>Auto 7597421</t>
   </si>
   <si>
     <t>In-Store P&amp;C Manager_NEW</t>
@@ -532,13 +517,10 @@
     <t>Test10</t>
   </si>
   <si>
-    <t>10698075</t>
-  </si>
-  <si>
-    <t>Emmalee</t>
-  </si>
-  <si>
-    <t>Kertzmann</t>
+    <t>Isabella</t>
+  </si>
+  <si>
+    <t>West</t>
   </si>
   <si>
     <t>In-Store P&amp;C Supervisor_NEW</t>
@@ -553,13 +535,10 @@
     <t>Test11</t>
   </si>
   <si>
-    <t>10698076</t>
-  </si>
-  <si>
-    <t>Ella</t>
-  </si>
-  <si>
-    <t>Jakubowski</t>
+    <t>Caterina</t>
+  </si>
+  <si>
+    <t>Dooley</t>
   </si>
   <si>
     <t>Supervisor_NEW</t>
@@ -571,13 +550,10 @@
     <t>Test12</t>
   </si>
   <si>
-    <t>10698078</t>
-  </si>
-  <si>
-    <t>Noelia</t>
-  </si>
-  <si>
-    <t>Cormier</t>
+    <t>Maryjane</t>
+  </si>
+  <si>
+    <t>Dietrich</t>
   </si>
   <si>
     <t>Retail Assistant Cash Office_NEW</t>
@@ -589,19 +565,10 @@
     <t>Test13</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'Jared Monahan' Employee:{10698079}TimeoutError: locator.click: Timeout 30000ms exceeded.
-Call log:
-  [2m- waiting for locator('text=Onboarding Guide: Visual Merchandiser_NEW - Jared Monahan')[22m
-</t>
-  </si>
-  <si>
-    <t>Failed</t>
-  </si>
-  <si>
-    <t>Jared</t>
-  </si>
-  <si>
-    <t>Monahan</t>
+    <t>Ruben</t>
+  </si>
+  <si>
+    <t>Stehr</t>
   </si>
   <si>
     <t>Visual Merchandiser_NEW</t>
@@ -610,16 +577,10 @@
     <t>Test14</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'Declan West' Employee:{}TimeoutError: locator.click: Timeout 30000ms exceeded.
-Call log:
-  [2m- waiting for getByLabel('Work Shift')[22m
-</t>
-  </si>
-  <si>
-    <t>Declan</t>
-  </si>
-  <si>
-    <t>West</t>
+    <t>Dawson</t>
+  </si>
+  <si>
+    <t>Maggio</t>
   </si>
   <si>
     <t>Retail Assistant Stockroom_NEW</t>
@@ -631,14 +592,10 @@
     <t>Test15</t>
   </si>
   <si>
-    <t>Test failed for 'Ola Franecki' Employee: Errors and AlertsErrorPage Error- You have not entered an amount within the Compensation Guidelines.
-- Grade Profile is Missing     (Employee Compensation Event For Hire Employee)Alerts &amp; find failed Screenshot Path:-&gt;H:\WorkdaySuite_Playwright_latestcode/WorkdayFailedScreenshot/2025-03-21T14-37-45-106Z.png</t>
-  </si>
-  <si>
-    <t>Ola</t>
-  </si>
-  <si>
-    <t>Franecki</t>
+    <t>Nigel</t>
+  </si>
+  <si>
+    <t>McClure</t>
   </si>
   <si>
     <t>In-Store Visual Merchandising Supervisor_NEW</t>
@@ -737,7 +694,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -1560,7 +1517,7 @@
       </c>
       <c r="K2" s="17">
         <f t="shared" ref="K2:K16" ca="1" si="0">TODAY()-7</f>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L2" s="13" t="s">
         <v>74</v>
@@ -1591,7 +1548,7 @@
       </c>
       <c r="U2" s="22">
         <f t="shared" ref="U2:U16" ca="1" si="1">TODAY()-31</f>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V2" s="16" t="s">
         <v>84</v>
@@ -1637,15 +1594,15 @@
       </c>
       <c r="AJ2" s="17">
         <f t="shared" ref="AJ2:AL16" ca="1" si="2">TODAY()-31</f>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK2" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL2" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM2" s="22" t="str">
         <f t="shared" ref="AM2:AM16" si="3">AF2</f>
@@ -1674,7 +1631,7 @@
       </c>
       <c r="AU2" s="17">
         <f t="shared" ref="AU2:AU16" ca="1" si="4">TODAY()+7</f>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV2" s="13" t="s">
         <v>74</v>
@@ -1684,7 +1641,7 @@
       </c>
       <c r="AX2" s="30">
         <f t="array" aca="1" ref="AX2:AX16" ca="1">_xlfn.RANDARRAY(15,1,1023456789000,9999999999999,TRUE)</f>
-        <v>5879589174643</v>
+        <v>3685585667530</v>
       </c>
       <c r="AY2" s="17" t="s">
         <v>98</v>
@@ -1700,7 +1657,7 @@
       </c>
       <c r="BC2" s="31">
         <f t="array" aca="1" ref="BC2:BC16" ca="1">_xlfn.RANDARRAY(15,1,12345678,99999999,TRUE)</f>
-        <v>90217606</v>
+        <v>81465916</v>
       </c>
       <c r="BD2" s="17" t="s">
         <v>98</v>
@@ -1743,7 +1700,7 @@
       </c>
       <c r="BQ2" s="34">
         <f t="array" aca="1" ref="BQ2:BQ16" ca="1">_xlfn.RANDARRAY(15,1,12345,99999,TRUE)</f>
-        <v>24175</v>
+        <v>38620</v>
       </c>
       <c r="BR2" s="17">
         <v>44562</v>
@@ -1756,7 +1713,7 @@
       </c>
       <c r="BU2" s="22">
         <f t="shared" ref="BU2:BU16" ca="1" si="5">TODAY()+365</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV2" s="16" t="s">
         <v>109</v>
@@ -1770,19 +1727,19 @@
         <v>111</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>72</v>
+        <v>112</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E3" s="13" t="s">
         <v>74</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H3" s="15" t="s">
         <v>77</v>
@@ -1795,7 +1752,7 @@
       </c>
       <c r="K3" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L3" s="13" t="s">
         <v>74</v>
@@ -1826,19 +1783,19 @@
       </c>
       <c r="U3" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V3" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W3" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X3" s="24" t="s">
         <v>86</v>
       </c>
       <c r="Y3" s="24" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Z3" s="24" t="s">
         <v>88</v>
@@ -1872,25 +1829,25 @@
       </c>
       <c r="AJ3" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK3" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL3" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM3" s="22" t="str">
         <f t="shared" si="3"/>
         <v>N/A</v>
       </c>
       <c r="AN3" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO3" s="24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AP3" s="24" t="s">
         <v>94</v>
@@ -1909,7 +1866,7 @@
       </c>
       <c r="AU3" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV3" s="13" t="s">
         <v>74</v>
@@ -1919,7 +1876,7 @@
       </c>
       <c r="AX3" s="30">
         <f ca="1"/>
-        <v>9629308524529</v>
+        <v>3276584545764</v>
       </c>
       <c r="AY3" s="17" t="s">
         <v>98</v>
@@ -1935,7 +1892,7 @@
       </c>
       <c r="BC3" s="31">
         <f ca="1"/>
-        <v>32599431</v>
+        <v>87692791</v>
       </c>
       <c r="BD3" s="17" t="s">
         <v>98</v>
@@ -1978,7 +1935,7 @@
       </c>
       <c r="BQ3" s="34">
         <f ca="1"/>
-        <v>30782</v>
+        <v>89330</v>
       </c>
       <c r="BR3" s="17">
         <v>44562</v>
@@ -1991,7 +1948,7 @@
       </c>
       <c r="BU3" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV3" s="16" t="s">
         <v>109</v>
@@ -1999,14 +1956,9 @@
     </row>
     <row r="4" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="B4" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>72</v>
-      </c>
+      <c r="C4" s="11"/>
       <c r="D4" s="12" t="s">
         <v>121</v>
       </c>
@@ -2030,7 +1982,7 @@
       </c>
       <c r="K4" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L4" s="13" t="s">
         <v>74</v>
@@ -2061,19 +2013,19 @@
       </c>
       <c r="U4" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V4" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W4" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X4" s="24" t="s">
         <v>124</v>
       </c>
       <c r="Y4" s="24" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Z4" s="24" t="s">
         <v>125</v>
@@ -2095,7 +2047,7 @@
       </c>
       <c r="AF4" s="28">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AG4" s="16" t="s">
         <v>92</v>
@@ -2108,25 +2060,25 @@
       </c>
       <c r="AJ4" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK4" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL4" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM4" s="22">
         <f t="shared" ca="1" si="3"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AN4" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO4" s="24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AP4" s="24" t="s">
         <v>94</v>
@@ -2145,7 +2097,7 @@
       </c>
       <c r="AU4" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV4" s="13" t="s">
         <v>74</v>
@@ -2155,7 +2107,7 @@
       </c>
       <c r="AX4" s="30">
         <f ca="1"/>
-        <v>4535670695535</v>
+        <v>8801576696517</v>
       </c>
       <c r="AY4" s="17" t="s">
         <v>98</v>
@@ -2171,7 +2123,7 @@
       </c>
       <c r="BC4" s="31">
         <f ca="1"/>
-        <v>57464761</v>
+        <v>59944209</v>
       </c>
       <c r="BD4" s="17" t="s">
         <v>98</v>
@@ -2214,7 +2166,7 @@
       </c>
       <c r="BQ4" s="34">
         <f ca="1"/>
-        <v>41501</v>
+        <v>58285</v>
       </c>
       <c r="BR4" s="17">
         <v>44562</v>
@@ -2227,7 +2179,7 @@
       </c>
       <c r="BU4" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV4" s="16" t="s">
         <v>109</v>
@@ -2237,14 +2189,9 @@
       <c r="A5" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="11"/>
+      <c r="D5" s="12" t="s">
         <v>129</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>73</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>74</v>
@@ -2266,7 +2213,7 @@
       </c>
       <c r="K5" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L5" s="13" t="s">
         <v>74</v>
@@ -2297,7 +2244,7 @@
       </c>
       <c r="U5" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V5" s="16" t="s">
         <v>84</v>
@@ -2331,7 +2278,7 @@
       </c>
       <c r="AF5" s="28">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AG5" s="16" t="s">
         <v>92</v>
@@ -2344,19 +2291,19 @@
       </c>
       <c r="AJ5" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK5" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL5" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM5" s="22">
         <f t="shared" ca="1" si="3"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AN5" s="16">
         <v>92</v>
@@ -2381,7 +2328,7 @@
       </c>
       <c r="AU5" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV5" s="13" t="s">
         <v>74</v>
@@ -2391,7 +2338,7 @@
       </c>
       <c r="AX5" s="30">
         <f ca="1"/>
-        <v>6805196517561</v>
+        <v>6140828842973</v>
       </c>
       <c r="AY5" s="17" t="s">
         <v>98</v>
@@ -2407,7 +2354,7 @@
       </c>
       <c r="BC5" s="31">
         <f ca="1"/>
-        <v>70131589</v>
+        <v>32827739</v>
       </c>
       <c r="BD5" s="17" t="s">
         <v>98</v>
@@ -2450,7 +2397,7 @@
       </c>
       <c r="BQ5" s="34">
         <f ca="1"/>
-        <v>57465</v>
+        <v>93929</v>
       </c>
       <c r="BR5" s="17">
         <v>44562</v>
@@ -2463,7 +2410,7 @@
       </c>
       <c r="BU5" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV5" s="16" t="s">
         <v>109</v>
@@ -2473,12 +2420,7 @@
       <c r="A6" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>72</v>
-      </c>
+      <c r="C6" s="11"/>
       <c r="D6" s="12" t="s">
         <v>121</v>
       </c>
@@ -2486,10 +2428,10 @@
         <v>74</v>
       </c>
       <c r="F6" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="G6" s="14" t="s">
         <v>137</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>138</v>
       </c>
       <c r="H6" s="15" t="s">
         <v>77</v>
@@ -2502,7 +2444,7 @@
       </c>
       <c r="K6" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L6" s="13" t="s">
         <v>74</v>
@@ -2533,19 +2475,19 @@
       </c>
       <c r="U6" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V6" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W6" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X6" s="24" t="s">
         <v>86</v>
       </c>
       <c r="Y6" s="24" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="Z6" s="24" t="s">
         <v>88</v>
@@ -2579,25 +2521,25 @@
       </c>
       <c r="AJ6" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK6" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL6" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM6" s="22" t="str">
         <f t="shared" si="3"/>
         <v>N/A</v>
       </c>
       <c r="AN6" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO6" s="24" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AP6" s="24" t="s">
         <v>94</v>
@@ -2616,7 +2558,7 @@
       </c>
       <c r="AU6" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV6" s="13" t="s">
         <v>74</v>
@@ -2626,7 +2568,7 @@
       </c>
       <c r="AX6" s="30">
         <f ca="1"/>
-        <v>3129804546869</v>
+        <v>7349315343891</v>
       </c>
       <c r="AY6" s="17" t="s">
         <v>98</v>
@@ -2642,7 +2584,7 @@
       </c>
       <c r="BC6" s="31">
         <f ca="1"/>
-        <v>85197506</v>
+        <v>33693281</v>
       </c>
       <c r="BD6" s="17" t="s">
         <v>98</v>
@@ -2685,7 +2627,7 @@
       </c>
       <c r="BQ6" s="34">
         <f ca="1"/>
-        <v>34673</v>
+        <v>19934</v>
       </c>
       <c r="BR6" s="17">
         <v>44562</v>
@@ -2698,7 +2640,7 @@
       </c>
       <c r="BU6" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV6" s="16" t="s">
         <v>109</v>
@@ -2706,25 +2648,20 @@
     </row>
     <row r="7" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" s="11"/>
+      <c r="D7" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="G7" s="14" t="s">
         <v>142</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>144</v>
       </c>
       <c r="H7" s="15" t="s">
         <v>77</v>
@@ -2737,7 +2674,7 @@
       </c>
       <c r="K7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L7" s="13" t="s">
         <v>74</v>
@@ -2768,13 +2705,13 @@
       </c>
       <c r="U7" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V7" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W7" s="23" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="X7" s="24" t="s">
         <v>86</v>
@@ -2814,15 +2751,15 @@
       </c>
       <c r="AJ7" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK7" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL7" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM7" s="22" t="str">
         <f t="shared" si="3"/>
@@ -2838,10 +2775,10 @@
         <v>94</v>
       </c>
       <c r="AQ7" s="24" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AR7" s="19" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AS7" s="13" t="s">
         <v>90</v>
@@ -2851,7 +2788,7 @@
       </c>
       <c r="AU7" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV7" s="13" t="s">
         <v>74</v>
@@ -2861,7 +2798,7 @@
       </c>
       <c r="AX7" s="30">
         <f ca="1"/>
-        <v>3882424946312</v>
+        <v>3621529537223</v>
       </c>
       <c r="AY7" s="17" t="s">
         <v>98</v>
@@ -2877,7 +2814,7 @@
       </c>
       <c r="BC7" s="31">
         <f ca="1"/>
-        <v>89025441</v>
+        <v>14511938</v>
       </c>
       <c r="BD7" s="17" t="s">
         <v>98</v>
@@ -2920,7 +2857,7 @@
       </c>
       <c r="BQ7" s="34">
         <f ca="1"/>
-        <v>15689</v>
+        <v>56524</v>
       </c>
       <c r="BR7" s="17">
         <v>44562</v>
@@ -2933,7 +2870,7 @@
       </c>
       <c r="BU7" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV7" s="16" t="s">
         <v>109</v>
@@ -2941,25 +2878,21 @@
     </row>
     <row r="8" spans="1:74" s="35" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" s="36"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="37" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="F8" s="38" t="s">
+        <v>147</v>
+      </c>
+      <c r="G8" s="38" t="s">
         <v>148</v>
-      </c>
-      <c r="B8" s="36" t="s">
-        <v>149</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D8" s="37" t="s">
-        <v>73</v>
-      </c>
-      <c r="E8" s="34" t="s">
-        <v>74</v>
-      </c>
-      <c r="F8" s="38" t="s">
-        <v>150</v>
-      </c>
-      <c r="G8" s="38" t="s">
-        <v>151</v>
       </c>
       <c r="H8" s="39" t="s">
         <v>77</v>
@@ -2972,7 +2905,7 @@
       </c>
       <c r="K8" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L8" s="34" t="s">
         <v>74</v>
@@ -3003,19 +2936,19 @@
       </c>
       <c r="U8" s="46">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V8" s="40" t="s">
         <v>84</v>
       </c>
       <c r="W8" s="40" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="X8" s="47" t="s">
         <v>124</v>
       </c>
       <c r="Y8" s="47" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="Z8" s="47" t="s">
         <v>88</v>
@@ -3037,7 +2970,7 @@
       </c>
       <c r="AF8" s="50">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AG8" s="40" t="s">
         <v>92</v>
@@ -3050,19 +2983,19 @@
       </c>
       <c r="AJ8" s="41">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK8" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL8" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM8" s="46">
         <f t="shared" ca="1" si="3"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AN8" s="40">
         <v>92</v>
@@ -3074,10 +3007,10 @@
         <v>94</v>
       </c>
       <c r="AQ8" s="47" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AR8" s="43" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AS8" s="34" t="s">
         <v>90</v>
@@ -3087,7 +3020,7 @@
       </c>
       <c r="AU8" s="41">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV8" s="34" t="s">
         <v>74</v>
@@ -3097,7 +3030,7 @@
       </c>
       <c r="AX8" s="30">
         <f ca="1"/>
-        <v>9824543293334</v>
+        <v>3508206066558</v>
       </c>
       <c r="AY8" s="41" t="s">
         <v>98</v>
@@ -3113,7 +3046,7 @@
       </c>
       <c r="BC8" s="31">
         <f ca="1"/>
-        <v>18676007</v>
+        <v>78816507</v>
       </c>
       <c r="BD8" s="41" t="s">
         <v>98</v>
@@ -3156,7 +3089,7 @@
       </c>
       <c r="BQ8" s="34">
         <f ca="1"/>
-        <v>75678</v>
+        <v>63924</v>
       </c>
       <c r="BR8" s="41">
         <v>44562</v>
@@ -3169,7 +3102,7 @@
       </c>
       <c r="BU8" s="46">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV8" s="40" t="s">
         <v>109</v>
@@ -3177,25 +3110,21 @@
     </row>
     <row r="9" spans="1:74" s="35" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>72</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="37" t="s">
-        <v>73</v>
+        <v>129</v>
       </c>
       <c r="E9" s="34" t="s">
         <v>74</v>
       </c>
       <c r="F9" s="38" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="G9" s="38" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="H9" s="39" t="s">
         <v>77</v>
@@ -3208,7 +3137,7 @@
       </c>
       <c r="K9" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L9" s="34" t="s">
         <v>74</v>
@@ -3239,19 +3168,19 @@
       </c>
       <c r="U9" s="46">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V9" s="40" t="s">
         <v>84</v>
       </c>
       <c r="W9" s="40" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="X9" s="47" t="s">
         <v>86</v>
       </c>
       <c r="Y9" s="47" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="Z9" s="47" t="s">
         <v>125</v>
@@ -3285,15 +3214,15 @@
       </c>
       <c r="AJ9" s="41">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK9" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL9" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM9" s="46" t="str">
         <f t="shared" si="3"/>
@@ -3309,10 +3238,10 @@
         <v>94</v>
       </c>
       <c r="AQ9" s="47" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AR9" s="43" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AS9" s="34" t="s">
         <v>90</v>
@@ -3322,7 +3251,7 @@
       </c>
       <c r="AU9" s="41">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV9" s="34" t="s">
         <v>74</v>
@@ -3332,7 +3261,7 @@
       </c>
       <c r="AX9" s="30">
         <f ca="1"/>
-        <v>6574353571659</v>
+        <v>3874603468215</v>
       </c>
       <c r="AY9" s="41" t="s">
         <v>98</v>
@@ -3348,7 +3277,7 @@
       </c>
       <c r="BC9" s="31">
         <f ca="1"/>
-        <v>78589868</v>
+        <v>57432686</v>
       </c>
       <c r="BD9" s="41" t="s">
         <v>98</v>
@@ -3391,7 +3320,7 @@
       </c>
       <c r="BQ9" s="34">
         <f ca="1"/>
-        <v>51690</v>
+        <v>98286</v>
       </c>
       <c r="BR9" s="41">
         <v>44562</v>
@@ -3404,7 +3333,7 @@
       </c>
       <c r="BU9" s="46">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV9" s="40" t="s">
         <v>109</v>
@@ -3412,25 +3341,20 @@
     </row>
     <row r="10" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>72</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="C10" s="11"/>
       <c r="D10" s="12" t="s">
-        <v>73</v>
+        <v>129</v>
       </c>
       <c r="E10" s="13" t="s">
         <v>74</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="H10" s="15" t="s">
         <v>77</v>
@@ -3443,7 +3367,7 @@
       </c>
       <c r="K10" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L10" s="13" t="s">
         <v>74</v>
@@ -3474,19 +3398,19 @@
       </c>
       <c r="U10" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V10" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W10" s="23" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="X10" s="24" t="s">
         <v>86</v>
       </c>
       <c r="Y10" s="24" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="Z10" s="24" t="s">
         <v>88</v>
@@ -3520,15 +3444,15 @@
       </c>
       <c r="AJ10" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK10" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL10" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM10" s="22" t="str">
         <f t="shared" si="3"/>
@@ -3544,10 +3468,10 @@
         <v>94</v>
       </c>
       <c r="AQ10" s="24" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AR10" s="19" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AS10" s="13" t="s">
         <v>90</v>
@@ -3557,7 +3481,7 @@
       </c>
       <c r="AU10" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV10" s="13" t="s">
         <v>74</v>
@@ -3567,7 +3491,7 @@
       </c>
       <c r="AX10" s="30">
         <f ca="1"/>
-        <v>3850767557935</v>
+        <v>4474505969211</v>
       </c>
       <c r="AY10" s="17" t="s">
         <v>98</v>
@@ -3583,7 +3507,7 @@
       </c>
       <c r="BC10" s="31">
         <f ca="1"/>
-        <v>74805827</v>
+        <v>21966030</v>
       </c>
       <c r="BD10" s="17" t="s">
         <v>98</v>
@@ -3626,7 +3550,7 @@
       </c>
       <c r="BQ10" s="34">
         <f ca="1"/>
-        <v>84181</v>
+        <v>64701</v>
       </c>
       <c r="BR10" s="17">
         <v>44562</v>
@@ -3639,7 +3563,7 @@
       </c>
       <c r="BU10" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV10" s="16" t="s">
         <v>109</v>
@@ -3647,14 +3571,10 @@
     </row>
     <row r="11" spans="1:74" s="35" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>72</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
       <c r="D11" s="37" t="s">
         <v>121</v>
       </c>
@@ -3662,10 +3582,10 @@
         <v>74</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="H11" s="39" t="s">
         <v>77</v>
@@ -3678,7 +3598,7 @@
       </c>
       <c r="K11" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L11" s="34" t="s">
         <v>74</v>
@@ -3709,19 +3629,19 @@
       </c>
       <c r="U11" s="46">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V11" s="40" t="s">
         <v>84</v>
       </c>
       <c r="W11" s="40" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X11" s="47" t="s">
         <v>86</v>
       </c>
       <c r="Y11" s="47" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="Z11" s="47" t="s">
         <v>88</v>
@@ -3755,31 +3675,31 @@
       </c>
       <c r="AJ11" s="41">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK11" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL11" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM11" s="46" t="str">
         <f t="shared" si="3"/>
         <v>N/A</v>
       </c>
       <c r="AN11" s="40" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO11" s="47" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="AP11" s="47" t="s">
         <v>94</v>
       </c>
       <c r="AQ11" s="47" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="AR11" s="43" t="s">
         <v>96</v>
@@ -3792,7 +3712,7 @@
       </c>
       <c r="AU11" s="41">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV11" s="34" t="s">
         <v>74</v>
@@ -3802,7 +3722,7 @@
       </c>
       <c r="AX11" s="30">
         <f ca="1"/>
-        <v>8820339871414</v>
+        <v>8301372478441</v>
       </c>
       <c r="AY11" s="41" t="s">
         <v>98</v>
@@ -3818,7 +3738,7 @@
       </c>
       <c r="BC11" s="31">
         <f ca="1"/>
-        <v>14120630</v>
+        <v>26107089</v>
       </c>
       <c r="BD11" s="41" t="s">
         <v>98</v>
@@ -3861,7 +3781,7 @@
       </c>
       <c r="BQ11" s="34">
         <f ca="1"/>
-        <v>56854</v>
+        <v>65536</v>
       </c>
       <c r="BR11" s="41">
         <v>44562</v>
@@ -3874,7 +3794,7 @@
       </c>
       <c r="BU11" s="46">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV11" s="40" t="s">
         <v>109</v>
@@ -3882,14 +3802,9 @@
     </row>
     <row r="12" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>72</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="C12" s="11"/>
       <c r="D12" s="12" t="s">
         <v>121</v>
       </c>
@@ -3897,10 +3812,10 @@
         <v>74</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="H12" s="15" t="s">
         <v>77</v>
@@ -3913,7 +3828,7 @@
       </c>
       <c r="K12" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L12" s="13" t="s">
         <v>74</v>
@@ -3944,19 +3859,19 @@
       </c>
       <c r="U12" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V12" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W12" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X12" s="24" t="s">
         <v>86</v>
       </c>
       <c r="Y12" s="24" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="Z12" s="24" t="s">
         <v>125</v>
@@ -3990,31 +3905,31 @@
       </c>
       <c r="AJ12" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK12" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL12" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM12" s="22" t="str">
         <f t="shared" si="3"/>
         <v>N/A</v>
       </c>
       <c r="AN12" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO12" s="24" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="AP12" s="24" t="s">
         <v>94</v>
       </c>
       <c r="AQ12" s="24" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="AR12" s="19" t="s">
         <v>96</v>
@@ -4027,7 +3942,7 @@
       </c>
       <c r="AU12" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV12" s="13" t="s">
         <v>74</v>
@@ -4037,7 +3952,7 @@
       </c>
       <c r="AX12" s="30">
         <f ca="1"/>
-        <v>6329089829318</v>
+        <v>8071851508394</v>
       </c>
       <c r="AY12" s="17" t="s">
         <v>98</v>
@@ -4053,7 +3968,7 @@
       </c>
       <c r="BC12" s="31">
         <f ca="1"/>
-        <v>44951213</v>
+        <v>33545930</v>
       </c>
       <c r="BD12" s="17" t="s">
         <v>98</v>
@@ -4096,7 +4011,7 @@
       </c>
       <c r="BQ12" s="34">
         <f ca="1"/>
-        <v>35567</v>
+        <v>69630</v>
       </c>
       <c r="BR12" s="17">
         <v>44562</v>
@@ -4109,7 +4024,7 @@
       </c>
       <c r="BU12" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV12" s="16" t="s">
         <v>109</v>
@@ -4117,14 +4032,10 @@
     </row>
     <row r="13" spans="1:74" s="35" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>72</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
       <c r="D13" s="37" t="s">
         <v>121</v>
       </c>
@@ -4132,10 +4043,10 @@
         <v>74</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="G13" s="38" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="H13" s="39" t="s">
         <v>77</v>
@@ -4148,7 +4059,7 @@
       </c>
       <c r="K13" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L13" s="34" t="s">
         <v>74</v>
@@ -4179,19 +4090,19 @@
       </c>
       <c r="U13" s="46">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V13" s="40" t="s">
         <v>84</v>
       </c>
       <c r="W13" s="40" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X13" s="47" t="s">
         <v>124</v>
       </c>
       <c r="Y13" s="47" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="Z13" s="47" t="s">
         <v>125</v>
@@ -4213,7 +4124,7 @@
       </c>
       <c r="AF13" s="50">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AG13" s="40" t="s">
         <v>92</v>
@@ -4226,25 +4137,25 @@
       </c>
       <c r="AJ13" s="41">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK13" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL13" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM13" s="46">
         <f t="shared" ca="1" si="3"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AN13" s="40" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO13" s="47" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="AP13" s="47" t="s">
         <v>94</v>
@@ -4263,7 +4174,7 @@
       </c>
       <c r="AU13" s="41">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV13" s="34" t="s">
         <v>74</v>
@@ -4273,7 +4184,7 @@
       </c>
       <c r="AX13" s="30">
         <f ca="1"/>
-        <v>3437783974897</v>
+        <v>2601554379503</v>
       </c>
       <c r="AY13" s="41" t="s">
         <v>98</v>
@@ -4289,7 +4200,7 @@
       </c>
       <c r="BC13" s="31">
         <f ca="1"/>
-        <v>64831588</v>
+        <v>29368358</v>
       </c>
       <c r="BD13" s="41" t="s">
         <v>98</v>
@@ -4332,7 +4243,7 @@
       </c>
       <c r="BQ13" s="34">
         <f ca="1"/>
-        <v>18196</v>
+        <v>63503</v>
       </c>
       <c r="BR13" s="41">
         <v>44562</v>
@@ -4345,7 +4256,7 @@
       </c>
       <c r="BU13" s="46">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV13" s="40" t="s">
         <v>109</v>
@@ -4353,14 +4264,10 @@
     </row>
     <row r="14" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>187</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="B14" s="10"/>
+      <c r="C14" s="11"/>
       <c r="D14" s="12" t="s">
         <v>121</v>
       </c>
@@ -4368,10 +4275,10 @@
         <v>74</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="H14" s="15" t="s">
         <v>77</v>
@@ -4384,7 +4291,7 @@
       </c>
       <c r="K14" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L14" s="13" t="s">
         <v>74</v>
@@ -4415,19 +4322,19 @@
       </c>
       <c r="U14" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V14" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W14" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X14" s="24" t="s">
         <v>124</v>
       </c>
       <c r="Y14" s="24" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="Z14" s="24" t="s">
         <v>88</v>
@@ -4449,7 +4356,7 @@
       </c>
       <c r="AF14" s="28">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AG14" s="16" t="s">
         <v>92</v>
@@ -4462,25 +4369,25 @@
       </c>
       <c r="AJ14" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK14" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL14" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM14" s="22">
         <f t="shared" ca="1" si="3"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AN14" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO14" s="24" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AP14" s="24" t="s">
         <v>94</v>
@@ -4499,7 +4406,7 @@
       </c>
       <c r="AU14" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV14" s="13" t="s">
         <v>74</v>
@@ -4509,7 +4416,7 @@
       </c>
       <c r="AX14" s="30">
         <f ca="1"/>
-        <v>3941794048959</v>
+        <v>8862074638158</v>
       </c>
       <c r="AY14" s="17" t="s">
         <v>98</v>
@@ -4525,7 +4432,7 @@
       </c>
       <c r="BC14" s="31">
         <f ca="1"/>
-        <v>82567804</v>
+        <v>86306078</v>
       </c>
       <c r="BD14" s="17" t="s">
         <v>98</v>
@@ -4568,7 +4475,7 @@
       </c>
       <c r="BQ14" s="34">
         <f ca="1"/>
-        <v>35646</v>
+        <v>32606</v>
       </c>
       <c r="BR14" s="17">
         <v>44562</v>
@@ -4581,7 +4488,7 @@
       </c>
       <c r="BU14" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV14" s="16" t="s">
         <v>109</v>
@@ -4589,14 +4496,9 @@
     </row>
     <row r="15" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>187</v>
-      </c>
+        <v>181</v>
+      </c>
+      <c r="C15" s="11"/>
       <c r="D15" s="12" t="s">
         <v>121</v>
       </c>
@@ -4604,10 +4506,10 @@
         <v>74</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="H15" s="15" t="s">
         <v>77</v>
@@ -4620,7 +4522,7 @@
       </c>
       <c r="K15" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L15" s="13" t="s">
         <v>74</v>
@@ -4651,19 +4553,19 @@
       </c>
       <c r="U15" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V15" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W15" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X15" s="24" t="s">
         <v>86</v>
       </c>
       <c r="Y15" s="24" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="Z15" s="24" t="s">
         <v>125</v>
@@ -4697,25 +4599,25 @@
       </c>
       <c r="AJ15" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK15" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL15" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM15" s="22" t="str">
         <f t="shared" si="3"/>
         <v>N/A</v>
       </c>
       <c r="AN15" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO15" s="24" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="AP15" s="24" t="s">
         <v>94</v>
@@ -4734,7 +4636,7 @@
       </c>
       <c r="AU15" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV15" s="13" t="s">
         <v>74</v>
@@ -4744,7 +4646,7 @@
       </c>
       <c r="AX15" s="30">
         <f ca="1"/>
-        <v>6519217663694</v>
+        <v>3201856004603</v>
       </c>
       <c r="AY15" s="17" t="s">
         <v>98</v>
@@ -4760,7 +4662,7 @@
       </c>
       <c r="BC15" s="31">
         <f ca="1"/>
-        <v>61320857</v>
+        <v>94568555</v>
       </c>
       <c r="BD15" s="17" t="s">
         <v>98</v>
@@ -4803,7 +4705,7 @@
       </c>
       <c r="BQ15" s="34">
         <f ca="1"/>
-        <v>75176</v>
+        <v>95267</v>
       </c>
       <c r="BR15" s="17">
         <v>44562</v>
@@ -4816,7 +4718,7 @@
       </c>
       <c r="BU15" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV15" s="16" t="s">
         <v>109</v>
@@ -4824,14 +4726,10 @@
     </row>
     <row r="16" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>187</v>
-      </c>
+        <v>186</v>
+      </c>
+      <c r="B16" s="10"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="12" t="s">
         <v>121</v>
       </c>
@@ -4839,10 +4737,10 @@
         <v>74</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>77</v>
@@ -4855,7 +4753,7 @@
       </c>
       <c r="K16" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L16" s="13" t="s">
         <v>74</v>
@@ -4886,19 +4784,19 @@
       </c>
       <c r="U16" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V16" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W16" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X16" s="24" t="s">
         <v>86</v>
       </c>
       <c r="Y16" s="24" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="Z16" s="24" t="s">
         <v>88</v>
@@ -4932,31 +4830,31 @@
       </c>
       <c r="AJ16" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK16" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL16" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM16" s="22" t="str">
         <f t="shared" si="3"/>
         <v>N/A</v>
       </c>
       <c r="AN16" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO16" s="24" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AP16" s="24" t="s">
         <v>94</v>
       </c>
       <c r="AQ16" s="24" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="AR16" s="19" t="s">
         <v>96</v>
@@ -4969,7 +4867,7 @@
       </c>
       <c r="AU16" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV16" s="13" t="s">
         <v>74</v>
@@ -4979,7 +4877,7 @@
       </c>
       <c r="AX16" s="30">
         <f ca="1"/>
-        <v>5300785576112</v>
+        <v>1348904031879</v>
       </c>
       <c r="AY16" s="17" t="s">
         <v>98</v>
@@ -4995,7 +4893,7 @@
       </c>
       <c r="BC16" s="31">
         <f ca="1"/>
-        <v>85925571</v>
+        <v>35193303</v>
       </c>
       <c r="BD16" s="17" t="s">
         <v>98</v>
@@ -5038,7 +4936,7 @@
       </c>
       <c r="BQ16" s="34">
         <f ca="1"/>
-        <v>46500</v>
+        <v>38041</v>
       </c>
       <c r="BR16" s="17">
         <v>44562</v>
@@ -5051,17 +4949,17 @@
       </c>
       <c r="BU16" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV16" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="17" spans="32:38" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="32:38" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AF17" s="54"/>
       <c r="AL17" s="17"/>
     </row>
-    <row r="18" spans="32:38" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="32:38" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AL18" s="17"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
code added for France
</commit_message>
<xml_diff>
--- a/Data/Hires/TestDataSloveniaMKv1.xlsx
+++ b/Data/Hires/TestDataSloveniaMKv1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{3BDC4FFC-8847-4F75-A8A0-26E78603E1E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{010A94B2-E573-40BF-B6FF-36154ED89136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="912" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="191">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -244,190 +244,190 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10698062</t>
+    <t>Test failed for 'Eden Rogahn' Employee: Errors and AlertsErrorsPage ErrorSorry, the data you requested could not be found. Please refresh your page.ErrorAllowance Amount is required.ErrorAllowance Amount is required.Alerts &amp; find failed Screenshot Path:-&gt;H:\WorkdaySuite_Playwright_MK/WorkdayFailedScreenshot/2025-03-25T10-19-24-088Z.png</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>795 Store Management (Zogop Dogegy (On Leave) (10185858))</t>
+  </si>
+  <si>
+    <t>Slovenia</t>
+  </si>
+  <si>
+    <t>Eden</t>
+  </si>
+  <si>
+    <t>Rogahn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">070-417-626 </t>
+  </si>
+  <si>
+    <t>Landline</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>Automation Street Name</t>
+  </si>
+  <si>
+    <t>Ljubljana</t>
+  </si>
+  <si>
+    <t>Street Address</t>
+  </si>
+  <si>
+    <t>Test@email.com</t>
+  </si>
+  <si>
+    <t>New Hire</t>
+  </si>
+  <si>
+    <t>Auto 9148281</t>
+  </si>
+  <si>
+    <t>Permanent</t>
+  </si>
+  <si>
+    <t>Store Manager_NEW</t>
+  </si>
+  <si>
+    <t>Full time</t>
+  </si>
+  <si>
+    <t>Salary</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>5 Days (Slovenia)</t>
+  </si>
+  <si>
+    <t>0- Ne gre za zaposlitev po ZUTD-A ali ZIUPTDSV</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Collective Agreement - Slovenia (01/01/1900 - )</t>
+  </si>
+  <si>
+    <t>Asistent v prodaji</t>
+  </si>
+  <si>
+    <t>IV.</t>
+  </si>
+  <si>
+    <t>Unique Master Citizen Number</t>
+  </si>
+  <si>
+    <t>01/01/1999</t>
+  </si>
+  <si>
+    <t>01/01/2045</t>
+  </si>
+  <si>
+    <t>Slovenia Tax Number</t>
+  </si>
+  <si>
+    <t>01/01/2041</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Citizen (Slovenia)</t>
+  </si>
+  <si>
+    <t>TestBankOFSlovenia</t>
+  </si>
+  <si>
+    <t>Checking</t>
+  </si>
+  <si>
+    <t>SI56 2633 0001 2039 086</t>
+  </si>
+  <si>
+    <t>Grun Frun</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>SVN Monthly</t>
+  </si>
+  <si>
+    <t>Test2</t>
+  </si>
+  <si>
+    <t>10698135</t>
   </si>
   <si>
     <t>Passed</t>
   </si>
   <si>
+    <t>795 Recruitment (Zosig Depazi (10280602))</t>
+  </si>
+  <si>
+    <t>Carmel</t>
+  </si>
+  <si>
+    <t>Hane</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Retail Assistant_NEW</t>
+  </si>
+  <si>
+    <t>94 Retail Operatives</t>
+  </si>
+  <si>
+    <t>01 Accessories</t>
+  </si>
+  <si>
+    <t>Test3</t>
+  </si>
+  <si>
+    <t>795 Retail Team 1 (Zogop Dogegy (10185858) (Inherited))</t>
+  </si>
+  <si>
+    <t>Jensen</t>
+  </si>
+  <si>
+    <t>O'Connell</t>
+  </si>
+  <si>
+    <t>Fixed Term (Fixed Term)</t>
+  </si>
+  <si>
+    <t>Part time</t>
+  </si>
+  <si>
+    <t>3 Days (Slovenia)</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Test4</t>
+  </si>
+  <si>
     <t>795 Store Management (Zogop Dogegy (10185858))</t>
   </si>
   <si>
-    <t>Slovenia</t>
-  </si>
-  <si>
-    <t>Parker</t>
-  </si>
-  <si>
-    <t>Halvorson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">070-417-626 </t>
-  </si>
-  <si>
-    <t>Landline</t>
-  </si>
-  <si>
-    <t>Home</t>
-  </si>
-  <si>
-    <t>Automation Street Name</t>
-  </si>
-  <si>
-    <t>Ljubljana</t>
-  </si>
-  <si>
-    <t>Street Address</t>
-  </si>
-  <si>
-    <t>Test@email.com</t>
-  </si>
-  <si>
-    <t>New Hire</t>
-  </si>
-  <si>
-    <t>Auto 95021107</t>
-  </si>
-  <si>
-    <t>Permanent</t>
-  </si>
-  <si>
-    <t>Store Manager_NEW</t>
-  </si>
-  <si>
-    <t>Full time</t>
-  </si>
-  <si>
-    <t>Salary</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>5 Days (Slovenia)</t>
-  </si>
-  <si>
-    <t>0- Ne gre za zaposlitev po ZUTD-A ali ZIUPTDSV</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Collective Agreement - Slovenia (01/01/1900 - )</t>
-  </si>
-  <si>
-    <t>Asistent v prodaji</t>
-  </si>
-  <si>
-    <t>IV.</t>
-  </si>
-  <si>
-    <t>Unique Master Citizen Number</t>
-  </si>
-  <si>
-    <t>01/01/1999</t>
-  </si>
-  <si>
-    <t>01/01/2045</t>
-  </si>
-  <si>
-    <t>Slovenia Tax Number</t>
-  </si>
-  <si>
-    <t>01/01/2041</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>Citizen (Slovenia)</t>
-  </si>
-  <si>
-    <t>TestBankOFSlovenia</t>
-  </si>
-  <si>
-    <t>Checking</t>
-  </si>
-  <si>
-    <t>SI56 2633 0001 2039 086</t>
-  </si>
-  <si>
-    <t>Grun Frun</t>
-  </si>
-  <si>
-    <t>Standard</t>
-  </si>
-  <si>
-    <t>SVN Monthly</t>
-  </si>
-  <si>
-    <t>Test2</t>
-  </si>
-  <si>
-    <t>10698063</t>
-  </si>
-  <si>
-    <t>795 Recruitment (Zosig Depazi (10280602))</t>
-  </si>
-  <si>
-    <t>Mittie</t>
-  </si>
-  <si>
-    <t>Tillman</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Retail Assistant_NEW</t>
-  </si>
-  <si>
-    <t>94 Retail Operatives</t>
-  </si>
-  <si>
-    <t>01 Accessories</t>
-  </si>
-  <si>
-    <t>Test3</t>
-  </si>
-  <si>
-    <t>10698065</t>
-  </si>
-  <si>
-    <t>795 Retail Team 1 (Zogop Dogegy (10185858) (Inherited))</t>
-  </si>
-  <si>
-    <t>Aurore</t>
-  </si>
-  <si>
-    <t>Kreiger</t>
-  </si>
-  <si>
-    <t>Fixed Term (Fixed Term)</t>
-  </si>
-  <si>
-    <t>Part time</t>
-  </si>
-  <si>
-    <t>3 Days (Slovenia)</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>Test4</t>
-  </si>
-  <si>
-    <t>10698066</t>
-  </si>
-  <si>
-    <t>Antwon</t>
-  </si>
-  <si>
-    <t>Johns</t>
-  </si>
-  <si>
-    <t>Auto 5780199</t>
+    <t>Jairo</t>
+  </si>
+  <si>
+    <t>Gerhold</t>
+  </si>
+  <si>
+    <t>Auto 13582723</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -439,13 +439,10 @@
     <t>Test5</t>
   </si>
   <si>
-    <t>10698068</t>
-  </si>
-  <si>
-    <t>Rebeka</t>
-  </si>
-  <si>
-    <t>Watsica</t>
+    <t>Fritz</t>
+  </si>
+  <si>
+    <t>Bayer</t>
   </si>
   <si>
     <t>In-Store Visual Merchandising Assistant_NEW</t>
@@ -457,16 +454,13 @@
     <t>Test6</t>
   </si>
   <si>
-    <t>10698070</t>
-  </si>
-  <si>
-    <t>Aron</t>
-  </si>
-  <si>
-    <t>Armstrong-McKenzie</t>
-  </si>
-  <si>
-    <t>Auto 7225502</t>
+    <t>Christopher</t>
+  </si>
+  <si>
+    <t>Schuppe</t>
+  </si>
+  <si>
+    <t>Auto 56790541</t>
   </si>
   <si>
     <t>Strokovni sodelavec v kadrovski službi</t>
@@ -478,16 +472,13 @@
     <t>Test7</t>
   </si>
   <si>
-    <t>10698072</t>
-  </si>
-  <si>
-    <t>Uriah</t>
-  </si>
-  <si>
-    <t>Medhurst</t>
-  </si>
-  <si>
-    <t>Auto 66154525</t>
+    <t>Bridget</t>
+  </si>
+  <si>
+    <t>Moen</t>
+  </si>
+  <si>
+    <t>Auto 67393007</t>
   </si>
   <si>
     <t>Assistant Store Manager_NEW</t>
@@ -496,16 +487,13 @@
     <t>Test8</t>
   </si>
   <si>
-    <t>10698073</t>
-  </si>
-  <si>
-    <t>Abby</t>
-  </si>
-  <si>
-    <t>Becker</t>
-  </si>
-  <si>
-    <t>Auto 6021389</t>
+    <t>Abdullah</t>
+  </si>
+  <si>
+    <t>Dickinson</t>
+  </si>
+  <si>
+    <t>Auto 39443903</t>
   </si>
   <si>
     <t>Department Manager_NEW</t>
@@ -514,16 +502,13 @@
     <t>Test9</t>
   </si>
   <si>
-    <t>10698074</t>
-  </si>
-  <si>
-    <t>Lindsey</t>
-  </si>
-  <si>
-    <t>Hagenes</t>
-  </si>
-  <si>
-    <t>Auto 51830818</t>
+    <t>Christa</t>
+  </si>
+  <si>
+    <t>Balistreri</t>
+  </si>
+  <si>
+    <t>Auto 7597421</t>
   </si>
   <si>
     <t>In-Store P&amp;C Manager_NEW</t>
@@ -532,13 +517,10 @@
     <t>Test10</t>
   </si>
   <si>
-    <t>10698075</t>
-  </si>
-  <si>
-    <t>Emmalee</t>
-  </si>
-  <si>
-    <t>Kertzmann</t>
+    <t>Isabella</t>
+  </si>
+  <si>
+    <t>West</t>
   </si>
   <si>
     <t>In-Store P&amp;C Supervisor_NEW</t>
@@ -553,13 +535,10 @@
     <t>Test11</t>
   </si>
   <si>
-    <t>10698076</t>
-  </si>
-  <si>
-    <t>Ella</t>
-  </si>
-  <si>
-    <t>Jakubowski</t>
+    <t>Caterina</t>
+  </si>
+  <si>
+    <t>Dooley</t>
   </si>
   <si>
     <t>Supervisor_NEW</t>
@@ -571,13 +550,10 @@
     <t>Test12</t>
   </si>
   <si>
-    <t>10698078</t>
-  </si>
-  <si>
-    <t>Noelia</t>
-  </si>
-  <si>
-    <t>Cormier</t>
+    <t>Maryjane</t>
+  </si>
+  <si>
+    <t>Dietrich</t>
   </si>
   <si>
     <t>Retail Assistant Cash Office_NEW</t>
@@ -589,19 +565,10 @@
     <t>Test13</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'Jared Monahan' Employee:{10698079}TimeoutError: locator.click: Timeout 30000ms exceeded.
-Call log:
-  [2m- waiting for locator('text=Onboarding Guide: Visual Merchandiser_NEW - Jared Monahan')[22m
-</t>
-  </si>
-  <si>
-    <t>Failed</t>
-  </si>
-  <si>
-    <t>Jared</t>
-  </si>
-  <si>
-    <t>Monahan</t>
+    <t>Ruben</t>
+  </si>
+  <si>
+    <t>Stehr</t>
   </si>
   <si>
     <t>Visual Merchandiser_NEW</t>
@@ -610,16 +577,10 @@
     <t>Test14</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'Declan West' Employee:{}TimeoutError: locator.click: Timeout 30000ms exceeded.
-Call log:
-  [2m- waiting for getByLabel('Work Shift')[22m
-</t>
-  </si>
-  <si>
-    <t>Declan</t>
-  </si>
-  <si>
-    <t>West</t>
+    <t>Dawson</t>
+  </si>
+  <si>
+    <t>Maggio</t>
   </si>
   <si>
     <t>Retail Assistant Stockroom_NEW</t>
@@ -631,14 +592,10 @@
     <t>Test15</t>
   </si>
   <si>
-    <t>Test failed for 'Ola Franecki' Employee: Errors and AlertsErrorPage Error- You have not entered an amount within the Compensation Guidelines.
-- Grade Profile is Missing     (Employee Compensation Event For Hire Employee)Alerts &amp; find failed Screenshot Path:-&gt;H:\WorkdaySuite_Playwright_latestcode/WorkdayFailedScreenshot/2025-03-21T14-37-45-106Z.png</t>
-  </si>
-  <si>
-    <t>Ola</t>
-  </si>
-  <si>
-    <t>Franecki</t>
+    <t>Nigel</t>
+  </si>
+  <si>
+    <t>McClure</t>
   </si>
   <si>
     <t>In-Store Visual Merchandising Supervisor_NEW</t>
@@ -737,7 +694,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -1560,7 +1517,7 @@
       </c>
       <c r="K2" s="17">
         <f t="shared" ref="K2:K16" ca="1" si="0">TODAY()-7</f>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L2" s="13" t="s">
         <v>74</v>
@@ -1591,7 +1548,7 @@
       </c>
       <c r="U2" s="22">
         <f t="shared" ref="U2:U16" ca="1" si="1">TODAY()-31</f>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V2" s="16" t="s">
         <v>84</v>
@@ -1637,15 +1594,15 @@
       </c>
       <c r="AJ2" s="17">
         <f t="shared" ref="AJ2:AL16" ca="1" si="2">TODAY()-31</f>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK2" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL2" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM2" s="22" t="str">
         <f t="shared" ref="AM2:AM16" si="3">AF2</f>
@@ -1674,7 +1631,7 @@
       </c>
       <c r="AU2" s="17">
         <f t="shared" ref="AU2:AU16" ca="1" si="4">TODAY()+7</f>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV2" s="13" t="s">
         <v>74</v>
@@ -1684,7 +1641,7 @@
       </c>
       <c r="AX2" s="30">
         <f t="array" aca="1" ref="AX2:AX16" ca="1">_xlfn.RANDARRAY(15,1,1023456789000,9999999999999,TRUE)</f>
-        <v>5879589174643</v>
+        <v>3685585667530</v>
       </c>
       <c r="AY2" s="17" t="s">
         <v>98</v>
@@ -1700,7 +1657,7 @@
       </c>
       <c r="BC2" s="31">
         <f t="array" aca="1" ref="BC2:BC16" ca="1">_xlfn.RANDARRAY(15,1,12345678,99999999,TRUE)</f>
-        <v>90217606</v>
+        <v>81465916</v>
       </c>
       <c r="BD2" s="17" t="s">
         <v>98</v>
@@ -1743,7 +1700,7 @@
       </c>
       <c r="BQ2" s="34">
         <f t="array" aca="1" ref="BQ2:BQ16" ca="1">_xlfn.RANDARRAY(15,1,12345,99999,TRUE)</f>
-        <v>24175</v>
+        <v>38620</v>
       </c>
       <c r="BR2" s="17">
         <v>44562</v>
@@ -1756,7 +1713,7 @@
       </c>
       <c r="BU2" s="22">
         <f t="shared" ref="BU2:BU16" ca="1" si="5">TODAY()+365</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV2" s="16" t="s">
         <v>109</v>
@@ -1770,19 +1727,19 @@
         <v>111</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>72</v>
+        <v>112</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E3" s="13" t="s">
         <v>74</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H3" s="15" t="s">
         <v>77</v>
@@ -1795,7 +1752,7 @@
       </c>
       <c r="K3" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L3" s="13" t="s">
         <v>74</v>
@@ -1826,19 +1783,19 @@
       </c>
       <c r="U3" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V3" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W3" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X3" s="24" t="s">
         <v>86</v>
       </c>
       <c r="Y3" s="24" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Z3" s="24" t="s">
         <v>88</v>
@@ -1872,25 +1829,25 @@
       </c>
       <c r="AJ3" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK3" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL3" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM3" s="22" t="str">
         <f t="shared" si="3"/>
         <v>N/A</v>
       </c>
       <c r="AN3" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO3" s="24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AP3" s="24" t="s">
         <v>94</v>
@@ -1909,7 +1866,7 @@
       </c>
       <c r="AU3" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV3" s="13" t="s">
         <v>74</v>
@@ -1919,7 +1876,7 @@
       </c>
       <c r="AX3" s="30">
         <f ca="1"/>
-        <v>9629308524529</v>
+        <v>3276584545764</v>
       </c>
       <c r="AY3" s="17" t="s">
         <v>98</v>
@@ -1935,7 +1892,7 @@
       </c>
       <c r="BC3" s="31">
         <f ca="1"/>
-        <v>32599431</v>
+        <v>87692791</v>
       </c>
       <c r="BD3" s="17" t="s">
         <v>98</v>
@@ -1978,7 +1935,7 @@
       </c>
       <c r="BQ3" s="34">
         <f ca="1"/>
-        <v>30782</v>
+        <v>89330</v>
       </c>
       <c r="BR3" s="17">
         <v>44562</v>
@@ -1991,7 +1948,7 @@
       </c>
       <c r="BU3" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV3" s="16" t="s">
         <v>109</v>
@@ -1999,14 +1956,9 @@
     </row>
     <row r="4" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="B4" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>72</v>
-      </c>
+      <c r="C4" s="11"/>
       <c r="D4" s="12" t="s">
         <v>121</v>
       </c>
@@ -2030,7 +1982,7 @@
       </c>
       <c r="K4" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L4" s="13" t="s">
         <v>74</v>
@@ -2061,19 +2013,19 @@
       </c>
       <c r="U4" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V4" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W4" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X4" s="24" t="s">
         <v>124</v>
       </c>
       <c r="Y4" s="24" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Z4" s="24" t="s">
         <v>125</v>
@@ -2095,7 +2047,7 @@
       </c>
       <c r="AF4" s="28">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AG4" s="16" t="s">
         <v>92</v>
@@ -2108,25 +2060,25 @@
       </c>
       <c r="AJ4" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK4" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL4" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM4" s="22">
         <f t="shared" ca="1" si="3"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AN4" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO4" s="24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AP4" s="24" t="s">
         <v>94</v>
@@ -2145,7 +2097,7 @@
       </c>
       <c r="AU4" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV4" s="13" t="s">
         <v>74</v>
@@ -2155,7 +2107,7 @@
       </c>
       <c r="AX4" s="30">
         <f ca="1"/>
-        <v>4535670695535</v>
+        <v>8801576696517</v>
       </c>
       <c r="AY4" s="17" t="s">
         <v>98</v>
@@ -2171,7 +2123,7 @@
       </c>
       <c r="BC4" s="31">
         <f ca="1"/>
-        <v>57464761</v>
+        <v>59944209</v>
       </c>
       <c r="BD4" s="17" t="s">
         <v>98</v>
@@ -2214,7 +2166,7 @@
       </c>
       <c r="BQ4" s="34">
         <f ca="1"/>
-        <v>41501</v>
+        <v>58285</v>
       </c>
       <c r="BR4" s="17">
         <v>44562</v>
@@ -2227,7 +2179,7 @@
       </c>
       <c r="BU4" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV4" s="16" t="s">
         <v>109</v>
@@ -2237,14 +2189,9 @@
       <c r="A5" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="11"/>
+      <c r="D5" s="12" t="s">
         <v>129</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>73</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>74</v>
@@ -2266,7 +2213,7 @@
       </c>
       <c r="K5" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L5" s="13" t="s">
         <v>74</v>
@@ -2297,7 +2244,7 @@
       </c>
       <c r="U5" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V5" s="16" t="s">
         <v>84</v>
@@ -2331,7 +2278,7 @@
       </c>
       <c r="AF5" s="28">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AG5" s="16" t="s">
         <v>92</v>
@@ -2344,19 +2291,19 @@
       </c>
       <c r="AJ5" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK5" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL5" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM5" s="22">
         <f t="shared" ca="1" si="3"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AN5" s="16">
         <v>92</v>
@@ -2381,7 +2328,7 @@
       </c>
       <c r="AU5" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV5" s="13" t="s">
         <v>74</v>
@@ -2391,7 +2338,7 @@
       </c>
       <c r="AX5" s="30">
         <f ca="1"/>
-        <v>6805196517561</v>
+        <v>6140828842973</v>
       </c>
       <c r="AY5" s="17" t="s">
         <v>98</v>
@@ -2407,7 +2354,7 @@
       </c>
       <c r="BC5" s="31">
         <f ca="1"/>
-        <v>70131589</v>
+        <v>32827739</v>
       </c>
       <c r="BD5" s="17" t="s">
         <v>98</v>
@@ -2450,7 +2397,7 @@
       </c>
       <c r="BQ5" s="34">
         <f ca="1"/>
-        <v>57465</v>
+        <v>93929</v>
       </c>
       <c r="BR5" s="17">
         <v>44562</v>
@@ -2463,7 +2410,7 @@
       </c>
       <c r="BU5" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV5" s="16" t="s">
         <v>109</v>
@@ -2473,12 +2420,7 @@
       <c r="A6" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>72</v>
-      </c>
+      <c r="C6" s="11"/>
       <c r="D6" s="12" t="s">
         <v>121</v>
       </c>
@@ -2486,10 +2428,10 @@
         <v>74</v>
       </c>
       <c r="F6" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="G6" s="14" t="s">
         <v>137</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>138</v>
       </c>
       <c r="H6" s="15" t="s">
         <v>77</v>
@@ -2502,7 +2444,7 @@
       </c>
       <c r="K6" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L6" s="13" t="s">
         <v>74</v>
@@ -2533,19 +2475,19 @@
       </c>
       <c r="U6" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V6" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W6" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X6" s="24" t="s">
         <v>86</v>
       </c>
       <c r="Y6" s="24" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="Z6" s="24" t="s">
         <v>88</v>
@@ -2579,25 +2521,25 @@
       </c>
       <c r="AJ6" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK6" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL6" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM6" s="22" t="str">
         <f t="shared" si="3"/>
         <v>N/A</v>
       </c>
       <c r="AN6" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO6" s="24" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AP6" s="24" t="s">
         <v>94</v>
@@ -2616,7 +2558,7 @@
       </c>
       <c r="AU6" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV6" s="13" t="s">
         <v>74</v>
@@ -2626,7 +2568,7 @@
       </c>
       <c r="AX6" s="30">
         <f ca="1"/>
-        <v>3129804546869</v>
+        <v>7349315343891</v>
       </c>
       <c r="AY6" s="17" t="s">
         <v>98</v>
@@ -2642,7 +2584,7 @@
       </c>
       <c r="BC6" s="31">
         <f ca="1"/>
-        <v>85197506</v>
+        <v>33693281</v>
       </c>
       <c r="BD6" s="17" t="s">
         <v>98</v>
@@ -2685,7 +2627,7 @@
       </c>
       <c r="BQ6" s="34">
         <f ca="1"/>
-        <v>34673</v>
+        <v>19934</v>
       </c>
       <c r="BR6" s="17">
         <v>44562</v>
@@ -2698,7 +2640,7 @@
       </c>
       <c r="BU6" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV6" s="16" t="s">
         <v>109</v>
@@ -2706,25 +2648,20 @@
     </row>
     <row r="7" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C7" s="11"/>
+      <c r="D7" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="G7" s="14" t="s">
         <v>142</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>144</v>
       </c>
       <c r="H7" s="15" t="s">
         <v>77</v>
@@ -2737,7 +2674,7 @@
       </c>
       <c r="K7" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L7" s="13" t="s">
         <v>74</v>
@@ -2768,13 +2705,13 @@
       </c>
       <c r="U7" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V7" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W7" s="23" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="X7" s="24" t="s">
         <v>86</v>
@@ -2814,15 +2751,15 @@
       </c>
       <c r="AJ7" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK7" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL7" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM7" s="22" t="str">
         <f t="shared" si="3"/>
@@ -2838,10 +2775,10 @@
         <v>94</v>
       </c>
       <c r="AQ7" s="24" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AR7" s="19" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AS7" s="13" t="s">
         <v>90</v>
@@ -2851,7 +2788,7 @@
       </c>
       <c r="AU7" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV7" s="13" t="s">
         <v>74</v>
@@ -2861,7 +2798,7 @@
       </c>
       <c r="AX7" s="30">
         <f ca="1"/>
-        <v>3882424946312</v>
+        <v>3621529537223</v>
       </c>
       <c r="AY7" s="17" t="s">
         <v>98</v>
@@ -2877,7 +2814,7 @@
       </c>
       <c r="BC7" s="31">
         <f ca="1"/>
-        <v>89025441</v>
+        <v>14511938</v>
       </c>
       <c r="BD7" s="17" t="s">
         <v>98</v>
@@ -2920,7 +2857,7 @@
       </c>
       <c r="BQ7" s="34">
         <f ca="1"/>
-        <v>15689</v>
+        <v>56524</v>
       </c>
       <c r="BR7" s="17">
         <v>44562</v>
@@ -2933,7 +2870,7 @@
       </c>
       <c r="BU7" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV7" s="16" t="s">
         <v>109</v>
@@ -2941,25 +2878,21 @@
     </row>
     <row r="8" spans="1:74" s="35" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" s="36"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="37" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="F8" s="38" t="s">
+        <v>147</v>
+      </c>
+      <c r="G8" s="38" t="s">
         <v>148</v>
-      </c>
-      <c r="B8" s="36" t="s">
-        <v>149</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="D8" s="37" t="s">
-        <v>73</v>
-      </c>
-      <c r="E8" s="34" t="s">
-        <v>74</v>
-      </c>
-      <c r="F8" s="38" t="s">
-        <v>150</v>
-      </c>
-      <c r="G8" s="38" t="s">
-        <v>151</v>
       </c>
       <c r="H8" s="39" t="s">
         <v>77</v>
@@ -2972,7 +2905,7 @@
       </c>
       <c r="K8" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L8" s="34" t="s">
         <v>74</v>
@@ -3003,19 +2936,19 @@
       </c>
       <c r="U8" s="46">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V8" s="40" t="s">
         <v>84</v>
       </c>
       <c r="W8" s="40" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="X8" s="47" t="s">
         <v>124</v>
       </c>
       <c r="Y8" s="47" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="Z8" s="47" t="s">
         <v>88</v>
@@ -3037,7 +2970,7 @@
       </c>
       <c r="AF8" s="50">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AG8" s="40" t="s">
         <v>92</v>
@@ -3050,19 +2983,19 @@
       </c>
       <c r="AJ8" s="41">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK8" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL8" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM8" s="46">
         <f t="shared" ca="1" si="3"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AN8" s="40">
         <v>92</v>
@@ -3074,10 +3007,10 @@
         <v>94</v>
       </c>
       <c r="AQ8" s="47" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AR8" s="43" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AS8" s="34" t="s">
         <v>90</v>
@@ -3087,7 +3020,7 @@
       </c>
       <c r="AU8" s="41">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV8" s="34" t="s">
         <v>74</v>
@@ -3097,7 +3030,7 @@
       </c>
       <c r="AX8" s="30">
         <f ca="1"/>
-        <v>9824543293334</v>
+        <v>3508206066558</v>
       </c>
       <c r="AY8" s="41" t="s">
         <v>98</v>
@@ -3113,7 +3046,7 @@
       </c>
       <c r="BC8" s="31">
         <f ca="1"/>
-        <v>18676007</v>
+        <v>78816507</v>
       </c>
       <c r="BD8" s="41" t="s">
         <v>98</v>
@@ -3156,7 +3089,7 @@
       </c>
       <c r="BQ8" s="34">
         <f ca="1"/>
-        <v>75678</v>
+        <v>63924</v>
       </c>
       <c r="BR8" s="41">
         <v>44562</v>
@@ -3169,7 +3102,7 @@
       </c>
       <c r="BU8" s="46">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV8" s="40" t="s">
         <v>109</v>
@@ -3177,25 +3110,21 @@
     </row>
     <row r="9" spans="1:74" s="35" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>72</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="37" t="s">
-        <v>73</v>
+        <v>129</v>
       </c>
       <c r="E9" s="34" t="s">
         <v>74</v>
       </c>
       <c r="F9" s="38" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="G9" s="38" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="H9" s="39" t="s">
         <v>77</v>
@@ -3208,7 +3137,7 @@
       </c>
       <c r="K9" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L9" s="34" t="s">
         <v>74</v>
@@ -3239,19 +3168,19 @@
       </c>
       <c r="U9" s="46">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V9" s="40" t="s">
         <v>84</v>
       </c>
       <c r="W9" s="40" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="X9" s="47" t="s">
         <v>86</v>
       </c>
       <c r="Y9" s="47" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="Z9" s="47" t="s">
         <v>125</v>
@@ -3285,15 +3214,15 @@
       </c>
       <c r="AJ9" s="41">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK9" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL9" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM9" s="46" t="str">
         <f t="shared" si="3"/>
@@ -3309,10 +3238,10 @@
         <v>94</v>
       </c>
       <c r="AQ9" s="47" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AR9" s="43" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AS9" s="34" t="s">
         <v>90</v>
@@ -3322,7 +3251,7 @@
       </c>
       <c r="AU9" s="41">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV9" s="34" t="s">
         <v>74</v>
@@ -3332,7 +3261,7 @@
       </c>
       <c r="AX9" s="30">
         <f ca="1"/>
-        <v>6574353571659</v>
+        <v>3874603468215</v>
       </c>
       <c r="AY9" s="41" t="s">
         <v>98</v>
@@ -3348,7 +3277,7 @@
       </c>
       <c r="BC9" s="31">
         <f ca="1"/>
-        <v>78589868</v>
+        <v>57432686</v>
       </c>
       <c r="BD9" s="41" t="s">
         <v>98</v>
@@ -3391,7 +3320,7 @@
       </c>
       <c r="BQ9" s="34">
         <f ca="1"/>
-        <v>51690</v>
+        <v>98286</v>
       </c>
       <c r="BR9" s="41">
         <v>44562</v>
@@ -3404,7 +3333,7 @@
       </c>
       <c r="BU9" s="46">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV9" s="40" t="s">
         <v>109</v>
@@ -3412,25 +3341,20 @@
     </row>
     <row r="10" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>72</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="C10" s="11"/>
       <c r="D10" s="12" t="s">
-        <v>73</v>
+        <v>129</v>
       </c>
       <c r="E10" s="13" t="s">
         <v>74</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="H10" s="15" t="s">
         <v>77</v>
@@ -3443,7 +3367,7 @@
       </c>
       <c r="K10" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L10" s="13" t="s">
         <v>74</v>
@@ -3474,19 +3398,19 @@
       </c>
       <c r="U10" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V10" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W10" s="23" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="X10" s="24" t="s">
         <v>86</v>
       </c>
       <c r="Y10" s="24" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="Z10" s="24" t="s">
         <v>88</v>
@@ -3520,15 +3444,15 @@
       </c>
       <c r="AJ10" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK10" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL10" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM10" s="22" t="str">
         <f t="shared" si="3"/>
@@ -3544,10 +3468,10 @@
         <v>94</v>
       </c>
       <c r="AQ10" s="24" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AR10" s="19" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="AS10" s="13" t="s">
         <v>90</v>
@@ -3557,7 +3481,7 @@
       </c>
       <c r="AU10" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV10" s="13" t="s">
         <v>74</v>
@@ -3567,7 +3491,7 @@
       </c>
       <c r="AX10" s="30">
         <f ca="1"/>
-        <v>3850767557935</v>
+        <v>4474505969211</v>
       </c>
       <c r="AY10" s="17" t="s">
         <v>98</v>
@@ -3583,7 +3507,7 @@
       </c>
       <c r="BC10" s="31">
         <f ca="1"/>
-        <v>74805827</v>
+        <v>21966030</v>
       </c>
       <c r="BD10" s="17" t="s">
         <v>98</v>
@@ -3626,7 +3550,7 @@
       </c>
       <c r="BQ10" s="34">
         <f ca="1"/>
-        <v>84181</v>
+        <v>64701</v>
       </c>
       <c r="BR10" s="17">
         <v>44562</v>
@@ -3639,7 +3563,7 @@
       </c>
       <c r="BU10" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV10" s="16" t="s">
         <v>109</v>
@@ -3647,14 +3571,10 @@
     </row>
     <row r="11" spans="1:74" s="35" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>72</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
       <c r="D11" s="37" t="s">
         <v>121</v>
       </c>
@@ -3662,10 +3582,10 @@
         <v>74</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="H11" s="39" t="s">
         <v>77</v>
@@ -3678,7 +3598,7 @@
       </c>
       <c r="K11" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L11" s="34" t="s">
         <v>74</v>
@@ -3709,19 +3629,19 @@
       </c>
       <c r="U11" s="46">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V11" s="40" t="s">
         <v>84</v>
       </c>
       <c r="W11" s="40" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X11" s="47" t="s">
         <v>86</v>
       </c>
       <c r="Y11" s="47" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="Z11" s="47" t="s">
         <v>88</v>
@@ -3755,31 +3675,31 @@
       </c>
       <c r="AJ11" s="41">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK11" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL11" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM11" s="46" t="str">
         <f t="shared" si="3"/>
         <v>N/A</v>
       </c>
       <c r="AN11" s="40" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO11" s="47" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="AP11" s="47" t="s">
         <v>94</v>
       </c>
       <c r="AQ11" s="47" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="AR11" s="43" t="s">
         <v>96</v>
@@ -3792,7 +3712,7 @@
       </c>
       <c r="AU11" s="41">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV11" s="34" t="s">
         <v>74</v>
@@ -3802,7 +3722,7 @@
       </c>
       <c r="AX11" s="30">
         <f ca="1"/>
-        <v>8820339871414</v>
+        <v>8301372478441</v>
       </c>
       <c r="AY11" s="41" t="s">
         <v>98</v>
@@ -3818,7 +3738,7 @@
       </c>
       <c r="BC11" s="31">
         <f ca="1"/>
-        <v>14120630</v>
+        <v>26107089</v>
       </c>
       <c r="BD11" s="41" t="s">
         <v>98</v>
@@ -3861,7 +3781,7 @@
       </c>
       <c r="BQ11" s="34">
         <f ca="1"/>
-        <v>56854</v>
+        <v>65536</v>
       </c>
       <c r="BR11" s="41">
         <v>44562</v>
@@ -3874,7 +3794,7 @@
       </c>
       <c r="BU11" s="46">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV11" s="40" t="s">
         <v>109</v>
@@ -3882,14 +3802,9 @@
     </row>
     <row r="12" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>72</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="C12" s="11"/>
       <c r="D12" s="12" t="s">
         <v>121</v>
       </c>
@@ -3897,10 +3812,10 @@
         <v>74</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="H12" s="15" t="s">
         <v>77</v>
@@ -3913,7 +3828,7 @@
       </c>
       <c r="K12" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L12" s="13" t="s">
         <v>74</v>
@@ -3944,19 +3859,19 @@
       </c>
       <c r="U12" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V12" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W12" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X12" s="24" t="s">
         <v>86</v>
       </c>
       <c r="Y12" s="24" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="Z12" s="24" t="s">
         <v>125</v>
@@ -3990,31 +3905,31 @@
       </c>
       <c r="AJ12" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK12" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL12" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM12" s="22" t="str">
         <f t="shared" si="3"/>
         <v>N/A</v>
       </c>
       <c r="AN12" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO12" s="24" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="AP12" s="24" t="s">
         <v>94</v>
       </c>
       <c r="AQ12" s="24" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="AR12" s="19" t="s">
         <v>96</v>
@@ -4027,7 +3942,7 @@
       </c>
       <c r="AU12" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV12" s="13" t="s">
         <v>74</v>
@@ -4037,7 +3952,7 @@
       </c>
       <c r="AX12" s="30">
         <f ca="1"/>
-        <v>6329089829318</v>
+        <v>8071851508394</v>
       </c>
       <c r="AY12" s="17" t="s">
         <v>98</v>
@@ -4053,7 +3968,7 @@
       </c>
       <c r="BC12" s="31">
         <f ca="1"/>
-        <v>44951213</v>
+        <v>33545930</v>
       </c>
       <c r="BD12" s="17" t="s">
         <v>98</v>
@@ -4096,7 +4011,7 @@
       </c>
       <c r="BQ12" s="34">
         <f ca="1"/>
-        <v>35567</v>
+        <v>69630</v>
       </c>
       <c r="BR12" s="17">
         <v>44562</v>
@@ -4109,7 +4024,7 @@
       </c>
       <c r="BU12" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV12" s="16" t="s">
         <v>109</v>
@@ -4117,14 +4032,10 @@
     </row>
     <row r="13" spans="1:74" s="35" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>72</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
       <c r="D13" s="37" t="s">
         <v>121</v>
       </c>
@@ -4132,10 +4043,10 @@
         <v>74</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="G13" s="38" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="H13" s="39" t="s">
         <v>77</v>
@@ -4148,7 +4059,7 @@
       </c>
       <c r="K13" s="41">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L13" s="34" t="s">
         <v>74</v>
@@ -4179,19 +4090,19 @@
       </c>
       <c r="U13" s="46">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V13" s="40" t="s">
         <v>84</v>
       </c>
       <c r="W13" s="40" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X13" s="47" t="s">
         <v>124</v>
       </c>
       <c r="Y13" s="47" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="Z13" s="47" t="s">
         <v>125</v>
@@ -4213,7 +4124,7 @@
       </c>
       <c r="AF13" s="50">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AG13" s="40" t="s">
         <v>92</v>
@@ -4226,25 +4137,25 @@
       </c>
       <c r="AJ13" s="41">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK13" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL13" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM13" s="46">
         <f t="shared" ca="1" si="3"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AN13" s="40" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO13" s="47" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="AP13" s="47" t="s">
         <v>94</v>
@@ -4263,7 +4174,7 @@
       </c>
       <c r="AU13" s="41">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV13" s="34" t="s">
         <v>74</v>
@@ -4273,7 +4184,7 @@
       </c>
       <c r="AX13" s="30">
         <f ca="1"/>
-        <v>3437783974897</v>
+        <v>2601554379503</v>
       </c>
       <c r="AY13" s="41" t="s">
         <v>98</v>
@@ -4289,7 +4200,7 @@
       </c>
       <c r="BC13" s="31">
         <f ca="1"/>
-        <v>64831588</v>
+        <v>29368358</v>
       </c>
       <c r="BD13" s="41" t="s">
         <v>98</v>
@@ -4332,7 +4243,7 @@
       </c>
       <c r="BQ13" s="34">
         <f ca="1"/>
-        <v>18196</v>
+        <v>63503</v>
       </c>
       <c r="BR13" s="41">
         <v>44562</v>
@@ -4345,7 +4256,7 @@
       </c>
       <c r="BU13" s="46">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV13" s="40" t="s">
         <v>109</v>
@@ -4353,14 +4264,10 @@
     </row>
     <row r="14" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>187</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="B14" s="10"/>
+      <c r="C14" s="11"/>
       <c r="D14" s="12" t="s">
         <v>121</v>
       </c>
@@ -4368,10 +4275,10 @@
         <v>74</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="H14" s="15" t="s">
         <v>77</v>
@@ -4384,7 +4291,7 @@
       </c>
       <c r="K14" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L14" s="13" t="s">
         <v>74</v>
@@ -4415,19 +4322,19 @@
       </c>
       <c r="U14" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V14" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W14" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X14" s="24" t="s">
         <v>124</v>
       </c>
       <c r="Y14" s="24" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="Z14" s="24" t="s">
         <v>88</v>
@@ -4449,7 +4356,7 @@
       </c>
       <c r="AF14" s="28">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AG14" s="16" t="s">
         <v>92</v>
@@ -4462,25 +4369,25 @@
       </c>
       <c r="AJ14" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK14" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL14" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM14" s="22">
         <f t="shared" ca="1" si="3"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="AN14" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO14" s="24" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AP14" s="24" t="s">
         <v>94</v>
@@ -4499,7 +4406,7 @@
       </c>
       <c r="AU14" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV14" s="13" t="s">
         <v>74</v>
@@ -4509,7 +4416,7 @@
       </c>
       <c r="AX14" s="30">
         <f ca="1"/>
-        <v>3941794048959</v>
+        <v>8862074638158</v>
       </c>
       <c r="AY14" s="17" t="s">
         <v>98</v>
@@ -4525,7 +4432,7 @@
       </c>
       <c r="BC14" s="31">
         <f ca="1"/>
-        <v>82567804</v>
+        <v>86306078</v>
       </c>
       <c r="BD14" s="17" t="s">
         <v>98</v>
@@ -4568,7 +4475,7 @@
       </c>
       <c r="BQ14" s="34">
         <f ca="1"/>
-        <v>35646</v>
+        <v>32606</v>
       </c>
       <c r="BR14" s="17">
         <v>44562</v>
@@ -4581,7 +4488,7 @@
       </c>
       <c r="BU14" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV14" s="16" t="s">
         <v>109</v>
@@ -4589,14 +4496,9 @@
     </row>
     <row r="15" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>187</v>
-      </c>
+        <v>181</v>
+      </c>
+      <c r="C15" s="11"/>
       <c r="D15" s="12" t="s">
         <v>121</v>
       </c>
@@ -4604,10 +4506,10 @@
         <v>74</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="H15" s="15" t="s">
         <v>77</v>
@@ -4620,7 +4522,7 @@
       </c>
       <c r="K15" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L15" s="13" t="s">
         <v>74</v>
@@ -4651,19 +4553,19 @@
       </c>
       <c r="U15" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V15" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W15" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X15" s="24" t="s">
         <v>86</v>
       </c>
       <c r="Y15" s="24" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="Z15" s="24" t="s">
         <v>125</v>
@@ -4697,25 +4599,25 @@
       </c>
       <c r="AJ15" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK15" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL15" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM15" s="22" t="str">
         <f t="shared" si="3"/>
         <v>N/A</v>
       </c>
       <c r="AN15" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO15" s="24" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="AP15" s="24" t="s">
         <v>94</v>
@@ -4734,7 +4636,7 @@
       </c>
       <c r="AU15" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV15" s="13" t="s">
         <v>74</v>
@@ -4744,7 +4646,7 @@
       </c>
       <c r="AX15" s="30">
         <f ca="1"/>
-        <v>6519217663694</v>
+        <v>3201856004603</v>
       </c>
       <c r="AY15" s="17" t="s">
         <v>98</v>
@@ -4760,7 +4662,7 @@
       </c>
       <c r="BC15" s="31">
         <f ca="1"/>
-        <v>61320857</v>
+        <v>94568555</v>
       </c>
       <c r="BD15" s="17" t="s">
         <v>98</v>
@@ -4803,7 +4705,7 @@
       </c>
       <c r="BQ15" s="34">
         <f ca="1"/>
-        <v>75176</v>
+        <v>95267</v>
       </c>
       <c r="BR15" s="17">
         <v>44562</v>
@@ -4816,7 +4718,7 @@
       </c>
       <c r="BU15" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV15" s="16" t="s">
         <v>109</v>
@@ -4824,14 +4726,10 @@
     </row>
     <row r="16" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>187</v>
-      </c>
+        <v>186</v>
+      </c>
+      <c r="B16" s="10"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="12" t="s">
         <v>121</v>
       </c>
@@ -4839,10 +4737,10 @@
         <v>74</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>77</v>
@@ -4855,7 +4753,7 @@
       </c>
       <c r="K16" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>45733</v>
+        <v>45734</v>
       </c>
       <c r="L16" s="13" t="s">
         <v>74</v>
@@ -4886,19 +4784,19 @@
       </c>
       <c r="U16" s="22">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="V16" s="16" t="s">
         <v>84</v>
       </c>
       <c r="W16" s="23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X16" s="24" t="s">
         <v>86</v>
       </c>
       <c r="Y16" s="24" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="Z16" s="24" t="s">
         <v>88</v>
@@ -4932,31 +4830,31 @@
       </c>
       <c r="AJ16" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AK16" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AL16" s="17">
         <f t="shared" ca="1" si="2"/>
-        <v>45709</v>
+        <v>45710</v>
       </c>
       <c r="AM16" s="22" t="str">
         <f t="shared" si="3"/>
         <v>N/A</v>
       </c>
       <c r="AN16" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AO16" s="24" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AP16" s="24" t="s">
         <v>94</v>
       </c>
       <c r="AQ16" s="24" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="AR16" s="19" t="s">
         <v>96</v>
@@ -4969,7 +4867,7 @@
       </c>
       <c r="AU16" s="17">
         <f t="shared" ca="1" si="4"/>
-        <v>45747</v>
+        <v>45748</v>
       </c>
       <c r="AV16" s="13" t="s">
         <v>74</v>
@@ -4979,7 +4877,7 @@
       </c>
       <c r="AX16" s="30">
         <f ca="1"/>
-        <v>5300785576112</v>
+        <v>1348904031879</v>
       </c>
       <c r="AY16" s="17" t="s">
         <v>98</v>
@@ -4995,7 +4893,7 @@
       </c>
       <c r="BC16" s="31">
         <f ca="1"/>
-        <v>85925571</v>
+        <v>35193303</v>
       </c>
       <c r="BD16" s="17" t="s">
         <v>98</v>
@@ -5038,7 +4936,7 @@
       </c>
       <c r="BQ16" s="34">
         <f ca="1"/>
-        <v>46500</v>
+        <v>38041</v>
       </c>
       <c r="BR16" s="17">
         <v>44562</v>
@@ -5051,17 +4949,17 @@
       </c>
       <c r="BU16" s="22">
         <f t="shared" ca="1" si="5"/>
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="BV16" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="17" spans="32:38" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="32:38" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AF17" s="54"/>
       <c r="AL17" s="17"/>
     </row>
-    <row r="18" spans="32:38" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="32:38" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AL18" s="17"/>
     </row>
   </sheetData>

</xml_diff>